<commit_message>
Update of the .xlsx files in the examples/ folder.
</commit_message>
<xml_diff>
--- a/examples/MPG-exten.xlsx
+++ b/examples/MPG-exten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dhv/git/pythmpg/git/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E62F93B-8916-E44B-98B7-83D054A28F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{414ED638-DAF6-CF40-882C-86AA28EE4F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6260" yWindow="840" windowWidth="22540" windowHeight="14900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -917,7 +917,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -975,10 +975,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1337,36 +1334,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1020" ht="14" x14ac:dyDescent="0.15">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>256</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
       <c r="E1" s="4"/>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>257</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
       <c r="L1" s="5"/>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="20" t="s">
         <v>255</v>
       </c>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
       <c r="Q1" s="5"/>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
     </row>
     <row r="2" spans="1:1020" ht="41.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="4"/>
@@ -9565,7 +9563,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:K1"/>
     <mergeCell ref="M1:P1"/>
-    <mergeCell ref="R1:V1"/>
+    <mergeCell ref="R1:W1"/>
   </mergeCells>
   <pageMargins left="0.55000000000000004" right="0.35" top="0.95" bottom="0.6" header="0.4" footer="0.511811023622047"/>
   <pageSetup fitToHeight="3" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>